<commit_message>
Update Mark Williamson OTJ Tracker.xlsx
</commit_message>
<xml_diff>
--- a/Mark Williamson OTJ Tracker.xlsx
+++ b/Mark Williamson OTJ Tracker.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="280">
   <si>
     <t xml:space="preserve">Apprenticeship Training Log </t>
   </si>
@@ -206,6 +206,12 @@
   </si>
   <si>
     <t xml:space="preserve">Snowflake Tutorial by Data Engineering Simplified Modules 6-8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google Cloud Platform – Associate Cloud Engineer Programme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K14, S14</t>
   </si>
   <si>
     <t xml:space="preserve">GRAND TOTAL</t>
@@ -2349,13 +2355,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>291600</xdr:colOff>
+      <xdr:colOff>291240</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>154800</xdr:rowOff>
+      <xdr:rowOff>154440</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="Picture 1" descr=""/>
+        <xdr:cNvPr id="1" name="Picture 1"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -2365,7 +2371,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="12153240" y="181080"/>
-          <a:ext cx="1266840" cy="1260720"/>
+          <a:ext cx="1266480" cy="1260360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2387,13 +2393,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>52200</xdr:colOff>
+      <xdr:colOff>51840</xdr:colOff>
       <xdr:row>32</xdr:row>
-      <xdr:rowOff>128520</xdr:rowOff>
+      <xdr:rowOff>128160</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Picture 2" descr=""/>
+        <xdr:cNvPr id="2" name="Picture 2"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -2403,7 +2409,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1030680" y="4953240"/>
-          <a:ext cx="12150000" cy="1605960"/>
+          <a:ext cx="12149640" cy="1605600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3301,7 +3307,7 @@
         <v>10</v>
       </c>
       <c r="D14" s="26" t="n">
-        <v>45980</v>
+        <v>46008</v>
       </c>
       <c r="E14" s="27" t="n">
         <v>21</v>
@@ -3358,7 +3364,7 @@
         <v>10</v>
       </c>
       <c r="D15" s="26" t="n">
-        <v>45980</v>
+        <v>46029</v>
       </c>
       <c r="E15" s="27" t="n">
         <v>18</v>
@@ -3411,8 +3417,12 @@
       <c r="B16" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
+      <c r="C16" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="26" t="n">
+        <v>46057</v>
+      </c>
       <c r="E16" s="27" t="n">
         <v>15</v>
       </c>
@@ -3421,7 +3431,7 @@
       </c>
       <c r="G16" s="22" t="n">
         <f aca="false">IF(NOT(ISBLANK(D16)), SUM(E16:F16), 0)</f>
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="H16" s="16"/>
       <c r="I16" s="29"/>
@@ -3464,8 +3474,12 @@
       <c r="B17" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="27"/>
-      <c r="D17" s="27"/>
+      <c r="C17" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" s="26" t="n">
+        <v>46092</v>
+      </c>
       <c r="E17" s="27" t="n">
         <v>15</v>
       </c>
@@ -3474,7 +3488,7 @@
       </c>
       <c r="G17" s="22" t="n">
         <f aca="false">IF(NOT(ISBLANK(D17)), SUM(E17:F17), 0)</f>
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="H17" s="16"/>
       <c r="I17" s="29"/>
@@ -3517,8 +3531,12 @@
       <c r="B18" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="27"/>
-      <c r="D18" s="27"/>
+      <c r="C18" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="26" t="n">
+        <v>46127</v>
+      </c>
       <c r="E18" s="27" t="n">
         <v>11</v>
       </c>
@@ -3527,7 +3545,7 @@
       </c>
       <c r="G18" s="22" t="n">
         <f aca="false">IF(NOT(ISBLANK(D18)), SUM(E18:F18), 0)</f>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H18" s="16"/>
       <c r="I18" s="29"/>
@@ -3582,7 +3600,7 @@
       </c>
       <c r="G19" s="36" t="n">
         <f aca="false">SUM(G6:G18)</f>
-        <v>302</v>
+        <v>367</v>
       </c>
       <c r="H19" s="16"/>
       <c r="I19" s="29"/>
@@ -4925,12 +4943,20 @@
     </row>
     <row r="46" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="14"/>
-      <c r="B46" s="30"/>
+      <c r="B46" s="30" t="s">
+        <v>58</v>
+      </c>
       <c r="C46" s="57"/>
-      <c r="D46" s="67"/>
-      <c r="E46" s="19"/>
+      <c r="D46" s="26" t="n">
+        <v>45746</v>
+      </c>
+      <c r="E46" s="19" t="s">
+        <v>59</v>
+      </c>
       <c r="F46" s="19"/>
-      <c r="G46" s="68"/>
+      <c r="G46" s="59" t="n">
+        <v>48</v>
+      </c>
       <c r="H46" s="54"/>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
@@ -5594,7 +5620,7 @@
       <c r="F61" s="74"/>
       <c r="G61" s="36" t="n">
         <f aca="false">SUM(G36:G60)</f>
-        <v>29.5</v>
+        <v>77.5</v>
       </c>
       <c r="H61" s="54"/>
       <c r="I61" s="2"/>
@@ -5679,7 +5705,7 @@
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="14"/>
       <c r="B63" s="78" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C63" s="78"/>
       <c r="D63" s="79"/>
@@ -5687,7 +5713,7 @@
       <c r="F63" s="80"/>
       <c r="G63" s="81" t="n">
         <f aca="false">G61+G19+G28+G62</f>
-        <v>403.5</v>
+        <v>516.5</v>
       </c>
       <c r="H63" s="82"/>
       <c r="I63" s="2"/>
@@ -5814,7 +5840,7 @@
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="14"/>
       <c r="B66" s="27" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C66" s="27" t="n">
         <v>359</v>
@@ -5861,11 +5887,11 @@
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="14"/>
       <c r="B67" s="27" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C67" s="27" t="n">
         <f aca="false">G63</f>
-        <v>403.5</v>
+        <v>516.5</v>
       </c>
       <c r="D67" s="2"/>
       <c r="F67" s="2"/>
@@ -5909,11 +5935,11 @@
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="14"/>
       <c r="B68" s="27" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C68" s="40" t="n">
         <f aca="false">C66-C67</f>
-        <v>-44.5</v>
+        <v>-157.5</v>
       </c>
       <c r="D68" s="2"/>
       <c r="F68" s="2"/>
@@ -11864,7 +11890,7 @@
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Please select from the list" errorStyle="stop" errorTitle="Invalid Entry!" operator="between" prompt="Please select from the list" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C16:C20 C33" type="list">
+    <dataValidation allowBlank="true" error="Please select from the list" errorStyle="stop" errorTitle="Invalid Entry!" operator="between" prompt="Please select from the list" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C19:C20 C33" type="list">
       <formula1>'List - Hide'!$D$2:$D$3</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -11903,78 +11929,78 @@
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="83" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="84" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C4" s="85" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="86" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C5" s="86"/>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="86" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C6" s="86"/>
     </row>
     <row r="7" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="86" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C7" s="86"/>
     </row>
     <row r="8" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="86" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C8" s="86" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="86" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C9" s="87" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="86" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C10" s="86" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="86" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C11" s="86" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="86" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C12" s="86" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="86" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C13" s="86" t="s">
         <v>10</v>
@@ -11982,15 +12008,15 @@
     </row>
     <row r="14" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="86" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C14" s="86" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="86" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C15" s="86"/>
     </row>
@@ -12091,24 +12117,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="89" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B1" s="49" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C1" s="49" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="90" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B2" s="91" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C2" s="92" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D2" s="69"/>
       <c r="E2" s="69"/>
@@ -12163,13 +12189,13 @@
     </row>
     <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="90" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B3" s="92" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C3" s="92" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D3" s="69"/>
       <c r="E3" s="69"/>
@@ -12224,13 +12250,13 @@
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="90" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B4" s="92" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C4" s="92" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D4" s="69"/>
       <c r="E4" s="69"/>
@@ -12285,13 +12311,13 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="90" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B5" s="92" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C5" s="92" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D5" s="69"/>
       <c r="E5" s="69"/>
@@ -12346,13 +12372,13 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="90" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B6" s="92" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C6" s="92" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D6" s="69"/>
       <c r="E6" s="69"/>
@@ -12407,13 +12433,13 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="90" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B7" s="92" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C7" s="92" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D7" s="69"/>
       <c r="E7" s="69"/>
@@ -12468,10 +12494,10 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="90" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B8" s="92" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C8" s="69"/>
       <c r="D8" s="69"/>
@@ -12527,10 +12553,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="90" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B9" s="92" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C9" s="69"/>
       <c r="D9" s="69"/>
@@ -12586,10 +12612,10 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="90" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B10" s="92" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C10" s="69"/>
       <c r="D10" s="69"/>
@@ -12645,10 +12671,10 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="90" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B11" s="92" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C11" s="69"/>
       <c r="D11" s="69"/>
@@ -12704,10 +12730,10 @@
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="90" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B12" s="69" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C12" s="69"/>
       <c r="D12" s="69"/>
@@ -12763,10 +12789,10 @@
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="90" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B13" s="69" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C13" s="69"/>
       <c r="D13" s="69"/>
@@ -12822,10 +12848,10 @@
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="90" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B14" s="69" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C14" s="69"/>
       <c r="D14" s="69"/>
@@ -12881,10 +12907,10 @@
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="90" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B15" s="69" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C15" s="69"/>
       <c r="D15" s="69"/>
@@ -12940,10 +12966,10 @@
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="90" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B16" s="69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C16" s="69"/>
       <c r="D16" s="69"/>
@@ -12999,10 +13025,10 @@
     </row>
     <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="90" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B17" s="69" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C17" s="69"/>
       <c r="D17" s="69"/>
@@ -13058,10 +13084,10 @@
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="90" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B18" s="69" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C18" s="69"/>
       <c r="D18" s="69"/>
@@ -13117,10 +13143,10 @@
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="90" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B19" s="69" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C19" s="69"/>
       <c r="D19" s="69"/>
@@ -13176,10 +13202,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="90" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B20" s="69" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C20" s="69"/>
       <c r="D20" s="69"/>
@@ -13235,10 +13261,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="90" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B21" s="69" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C21" s="69"/>
       <c r="D21" s="69"/>
@@ -13294,10 +13320,10 @@
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="90" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B22" s="69" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C22" s="69"/>
       <c r="D22" s="69"/>
@@ -13353,10 +13379,10 @@
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="90" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B23" s="69" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C23" s="69"/>
       <c r="D23" s="69"/>
@@ -13412,10 +13438,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="90" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B24" s="69" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C24" s="69"/>
       <c r="D24" s="69"/>
@@ -13471,10 +13497,10 @@
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="90" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B25" s="69" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C25" s="69"/>
       <c r="D25" s="69"/>
@@ -13530,10 +13556,10 @@
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="90" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B26" s="69" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C26" s="69"/>
       <c r="D26" s="69"/>
@@ -13589,10 +13615,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B27" s="69" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C27" s="69"/>
       <c r="D27" s="69"/>
@@ -13648,10 +13674,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="90" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B28" s="69" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C28" s="69"/>
       <c r="D28" s="69"/>
@@ -13707,10 +13733,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="90" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B29" s="69" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C29" s="69"/>
       <c r="D29" s="69"/>
@@ -13766,10 +13792,10 @@
     </row>
     <row r="30" s="90" customFormat="true" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="90" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B30" s="92" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C30" s="92"/>
       <c r="D30" s="92"/>
@@ -13825,7 +13851,7 @@
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="90" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B31" s="69"/>
       <c r="C31" s="69"/>
@@ -25489,10 +25515,10 @@
       <c r="B1" s="93"/>
       <c r="C1" s="93"/>
       <c r="D1" s="94" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E1" s="95" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F1" s="95" t="s">
         <v>11</v>
@@ -25531,28 +25557,28 @@
         <v>22</v>
       </c>
       <c r="R1" s="95" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="S1" s="95" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="T1" s="95" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U1" s="95" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="V1" s="95" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="W1" s="95" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="X1" s="95" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="Y1" s="96" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="Z1" s="93"/>
       <c r="AA1" s="93"/>
@@ -25566,13 +25592,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="97" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B2" s="98" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="99" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D2" s="100"/>
       <c r="E2" s="101" t="n">
@@ -25627,7 +25653,7 @@
       <c r="A3" s="97"/>
       <c r="B3" s="98"/>
       <c r="C3" s="104" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D3" s="105"/>
       <c r="E3" s="103"/>
@@ -25679,7 +25705,7 @@
       <c r="A4" s="97"/>
       <c r="B4" s="98"/>
       <c r="C4" s="104" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D4" s="105"/>
       <c r="E4" s="103"/>
@@ -25731,7 +25757,7 @@
       <c r="A5" s="97"/>
       <c r="B5" s="98"/>
       <c r="C5" s="104" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D5" s="105"/>
       <c r="E5" s="103"/>
@@ -25785,7 +25811,7 @@
         <v>2</v>
       </c>
       <c r="C6" s="104" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D6" s="105"/>
       <c r="E6" s="103"/>
@@ -25839,7 +25865,7 @@
       <c r="A7" s="97"/>
       <c r="B7" s="107"/>
       <c r="C7" s="104" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D7" s="105"/>
       <c r="E7" s="103"/>
@@ -25891,7 +25917,7 @@
       <c r="A8" s="97"/>
       <c r="B8" s="107"/>
       <c r="C8" s="104" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D8" s="105"/>
       <c r="E8" s="103"/>
@@ -25942,7 +25968,7 @@
       <c r="A9" s="97"/>
       <c r="B9" s="107"/>
       <c r="C9" s="104" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D9" s="105"/>
       <c r="E9" s="103"/>
@@ -25982,7 +26008,7 @@
       <c r="Z9" s="103"/>
       <c r="AA9" s="103"/>
       <c r="AB9" s="103" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="AC9" s="103" t="n">
         <f aca="false">E2</f>
@@ -26000,7 +26026,7 @@
         <v>3</v>
       </c>
       <c r="C10" s="104" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D10" s="105"/>
       <c r="E10" s="103"/>
@@ -26042,13 +26068,13 @@
       <c r="Z10" s="103"/>
       <c r="AA10" s="103"/>
       <c r="AB10" s="108" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="AC10" s="103"/>
       <c r="AD10" s="103"/>
       <c r="AE10" s="103"/>
       <c r="AF10" s="103" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="AG10" s="103"/>
       <c r="AH10" s="103"/>
@@ -26057,7 +26083,7 @@
       <c r="A11" s="97"/>
       <c r="B11" s="107"/>
       <c r="C11" s="104" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D11" s="105"/>
       <c r="E11" s="103"/>
@@ -26097,7 +26123,7 @@
       <c r="Z11" s="103"/>
       <c r="AA11" s="103"/>
       <c r="AB11" s="109" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="AC11" s="110" t="n">
         <f aca="false">Y79+AC9</f>
@@ -26113,7 +26139,7 @@
       <c r="A12" s="97"/>
       <c r="B12" s="107"/>
       <c r="C12" s="104" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D12" s="105"/>
       <c r="E12" s="103"/>
@@ -26154,16 +26180,16 @@
       <c r="AA12" s="103"/>
       <c r="AB12" s="103"/>
       <c r="AC12" s="111" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="AD12" s="111" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="AE12" s="112" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AF12" s="112" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="AG12" s="103"/>
       <c r="AH12" s="103"/>
@@ -26172,7 +26198,7 @@
       <c r="A13" s="97"/>
       <c r="B13" s="107"/>
       <c r="C13" s="104" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D13" s="105"/>
       <c r="E13" s="103"/>
@@ -26192,7 +26218,7 @@
       <c r="Q13" s="106"/>
       <c r="R13" s="103"/>
       <c r="S13" s="113" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="T13" s="103"/>
       <c r="U13" s="105" t="n">
@@ -26241,7 +26267,7 @@
         <v>4</v>
       </c>
       <c r="C14" s="104" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D14" s="105"/>
       <c r="E14" s="103"/>
@@ -26307,7 +26333,7 @@
       <c r="A15" s="97"/>
       <c r="B15" s="107"/>
       <c r="C15" s="104" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D15" s="105"/>
       <c r="E15" s="103"/>
@@ -26371,7 +26397,7 @@
       <c r="A16" s="97"/>
       <c r="B16" s="107"/>
       <c r="C16" s="104" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D16" s="105"/>
       <c r="E16" s="103"/>
@@ -26435,7 +26461,7 @@
       <c r="A17" s="97"/>
       <c r="B17" s="107"/>
       <c r="C17" s="104" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D17" s="105"/>
       <c r="E17" s="103"/>
@@ -26501,7 +26527,7 @@
         <v>5</v>
       </c>
       <c r="C18" s="104" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D18" s="105"/>
       <c r="E18" s="103"/>
@@ -26567,7 +26593,7 @@
       <c r="A19" s="97"/>
       <c r="B19" s="107"/>
       <c r="C19" s="104" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D19" s="105"/>
       <c r="E19" s="103"/>
@@ -26632,7 +26658,7 @@
       <c r="A20" s="97"/>
       <c r="B20" s="107"/>
       <c r="C20" s="104" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D20" s="105"/>
       <c r="E20" s="103"/>
@@ -26696,7 +26722,7 @@
       <c r="A21" s="97"/>
       <c r="B21" s="107"/>
       <c r="C21" s="104" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D21" s="105"/>
       <c r="E21" s="103"/>
@@ -26762,7 +26788,7 @@
         <v>6</v>
       </c>
       <c r="C22" s="104" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D22" s="105"/>
       <c r="E22" s="103"/>
@@ -26827,7 +26853,7 @@
       <c r="A23" s="97"/>
       <c r="B23" s="107"/>
       <c r="C23" s="104" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D23" s="105"/>
       <c r="E23" s="103"/>
@@ -26847,7 +26873,7 @@
       <c r="Q23" s="106"/>
       <c r="R23" s="103"/>
       <c r="S23" s="113" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="T23" s="103"/>
       <c r="U23" s="105" t="n">
@@ -26893,7 +26919,7 @@
       <c r="A24" s="97"/>
       <c r="B24" s="107"/>
       <c r="C24" s="104" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D24" s="105"/>
       <c r="E24" s="103"/>
@@ -26955,7 +26981,7 @@
       <c r="A25" s="97"/>
       <c r="B25" s="107"/>
       <c r="C25" s="104" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="D25" s="105"/>
       <c r="E25" s="103"/>
@@ -27016,7 +27042,7 @@
         <v>7</v>
       </c>
       <c r="C26" s="104" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D26" s="105"/>
       <c r="E26" s="103"/>
@@ -27060,13 +27086,13 @@
       <c r="AA26" s="103"/>
       <c r="AB26" s="93"/>
       <c r="AC26" s="111" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="AD26" s="111" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="AE26" s="112" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AF26" s="103"/>
       <c r="AG26" s="103"/>
@@ -27075,7 +27101,7 @@
       <c r="A27" s="97"/>
       <c r="B27" s="107"/>
       <c r="C27" s="104" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D27" s="105"/>
       <c r="E27" s="103"/>
@@ -27116,7 +27142,7 @@
       <c r="Z27" s="103"/>
       <c r="AA27" s="103"/>
       <c r="AB27" s="122" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="AC27" s="115" t="n">
         <v>10</v>
@@ -27132,7 +27158,7 @@
       <c r="A28" s="97"/>
       <c r="B28" s="107"/>
       <c r="C28" s="104" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D28" s="105"/>
       <c r="E28" s="103"/>
@@ -27173,7 +27199,7 @@
       <c r="Z28" s="103"/>
       <c r="AA28" s="103"/>
       <c r="AB28" s="122" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="AC28" s="115" t="n">
         <v>10</v>
@@ -27189,7 +27215,7 @@
       <c r="A29" s="97"/>
       <c r="B29" s="107"/>
       <c r="C29" s="104" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D29" s="105"/>
       <c r="E29" s="103"/>
@@ -27227,11 +27253,11 @@
         <v>7.5</v>
       </c>
       <c r="Z29" s="103" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="AA29" s="103"/>
       <c r="AB29" s="122" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="AC29" s="115" t="n">
         <v>10</v>
@@ -27249,7 +27275,7 @@
         <v>8</v>
       </c>
       <c r="C30" s="104" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D30" s="105"/>
       <c r="E30" s="103"/>
@@ -27290,7 +27316,7 @@
       </c>
       <c r="AA30" s="103"/>
       <c r="AB30" s="122" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="AC30" s="115" t="n">
         <v>10</v>
@@ -27306,7 +27332,7 @@
       <c r="A31" s="97"/>
       <c r="B31" s="107"/>
       <c r="C31" s="104" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D31" s="105"/>
       <c r="E31" s="103"/>
@@ -27346,7 +27372,7 @@
       <c r="Z31" s="103"/>
       <c r="AA31" s="103"/>
       <c r="AB31" s="122" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="AC31" s="118" t="n">
         <v>10</v>
@@ -27362,7 +27388,7 @@
       <c r="A32" s="97"/>
       <c r="B32" s="107"/>
       <c r="C32" s="104" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D32" s="105"/>
       <c r="E32" s="103"/>
@@ -27413,7 +27439,7 @@
       <c r="A33" s="97"/>
       <c r="B33" s="107"/>
       <c r="C33" s="104" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D33" s="105"/>
       <c r="E33" s="103"/>
@@ -27433,7 +27459,7 @@
       <c r="Q33" s="106"/>
       <c r="R33" s="103"/>
       <c r="S33" s="113" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="T33" s="103"/>
       <c r="U33" s="105" t="n">
@@ -27462,7 +27488,7 @@
         <v>9</v>
       </c>
       <c r="C34" s="104" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D34" s="105"/>
       <c r="E34" s="103"/>
@@ -27507,7 +27533,7 @@
       <c r="A35" s="97"/>
       <c r="B35" s="107"/>
       <c r="C35" s="104" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D35" s="105"/>
       <c r="E35" s="103"/>
@@ -27551,7 +27577,7 @@
       <c r="A36" s="97"/>
       <c r="B36" s="107"/>
       <c r="C36" s="104" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D36" s="105"/>
       <c r="E36" s="103"/>
@@ -27589,7 +27615,7 @@
         <v>7.5</v>
       </c>
       <c r="Z36" s="103" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="AA36" s="103"/>
     </row>
@@ -27597,7 +27623,7 @@
       <c r="A37" s="97"/>
       <c r="B37" s="107"/>
       <c r="C37" s="104" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D37" s="105"/>
       <c r="E37" s="103"/>
@@ -27643,7 +27669,7 @@
         <v>10</v>
       </c>
       <c r="C38" s="104" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D38" s="105"/>
       <c r="E38" s="103"/>
@@ -27690,7 +27716,7 @@
       <c r="A39" s="97"/>
       <c r="B39" s="107"/>
       <c r="C39" s="104" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D39" s="105"/>
       <c r="E39" s="103"/>
@@ -27736,7 +27762,7 @@
       <c r="A40" s="97"/>
       <c r="B40" s="107"/>
       <c r="C40" s="104" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D40" s="105"/>
       <c r="E40" s="103"/>
@@ -27781,7 +27807,7 @@
       <c r="A41" s="97"/>
       <c r="B41" s="107"/>
       <c r="C41" s="104" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D41" s="105"/>
       <c r="E41" s="103"/>
@@ -27834,7 +27860,7 @@
         <v>11</v>
       </c>
       <c r="C42" s="104" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D42" s="105"/>
       <c r="E42" s="103"/>
@@ -27886,7 +27912,7 @@
       <c r="A43" s="97"/>
       <c r="B43" s="107"/>
       <c r="C43" s="104" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D43" s="105"/>
       <c r="E43" s="103"/>
@@ -27906,7 +27932,7 @@
       <c r="Q43" s="106"/>
       <c r="R43" s="103"/>
       <c r="S43" s="113" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="T43" s="103"/>
       <c r="U43" s="105" t="n">
@@ -27940,7 +27966,7 @@
       <c r="A44" s="97"/>
       <c r="B44" s="107"/>
       <c r="C44" s="104" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D44" s="105"/>
       <c r="E44" s="103"/>
@@ -27991,7 +28017,7 @@
       <c r="A45" s="97"/>
       <c r="B45" s="107"/>
       <c r="C45" s="104" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D45" s="105"/>
       <c r="E45" s="103"/>
@@ -28044,7 +28070,7 @@
         <v>12</v>
       </c>
       <c r="C46" s="104" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D46" s="105"/>
       <c r="E46" s="103"/>
@@ -28097,7 +28123,7 @@
       <c r="A47" s="97"/>
       <c r="B47" s="107"/>
       <c r="C47" s="104" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D47" s="105"/>
       <c r="E47" s="103"/>
@@ -28148,7 +28174,7 @@
       <c r="A48" s="97"/>
       <c r="B48" s="107"/>
       <c r="C48" s="104" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D48" s="105"/>
       <c r="E48" s="103"/>
@@ -28186,7 +28212,7 @@
         <v>9.5</v>
       </c>
       <c r="Z48" s="103" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="AA48" s="103"/>
       <c r="AB48" s="103"/>
@@ -28201,7 +28227,7 @@
       <c r="A49" s="97"/>
       <c r="B49" s="107"/>
       <c r="C49" s="104" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D49" s="105"/>
       <c r="E49" s="103"/>
@@ -28254,7 +28280,7 @@
         <v>13</v>
       </c>
       <c r="C50" s="104" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D50" s="105"/>
       <c r="E50" s="103"/>
@@ -28307,7 +28333,7 @@
       <c r="A51" s="97"/>
       <c r="B51" s="107"/>
       <c r="C51" s="104" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D51" s="105"/>
       <c r="E51" s="103"/>
@@ -28358,7 +28384,7 @@
       <c r="A52" s="97"/>
       <c r="B52" s="107"/>
       <c r="C52" s="104" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D52" s="105"/>
       <c r="E52" s="103"/>
@@ -28408,7 +28434,7 @@
       <c r="A53" s="97"/>
       <c r="B53" s="107"/>
       <c r="C53" s="104" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D53" s="105"/>
       <c r="E53" s="103"/>
@@ -28461,7 +28487,7 @@
         <v>14</v>
       </c>
       <c r="C54" s="104" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="D54" s="105"/>
       <c r="E54" s="103"/>
@@ -28514,7 +28540,7 @@
       <c r="A55" s="97"/>
       <c r="B55" s="107"/>
       <c r="C55" s="104" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D55" s="105"/>
       <c r="E55" s="103"/>
@@ -28566,7 +28592,7 @@
       <c r="A56" s="97"/>
       <c r="B56" s="107"/>
       <c r="C56" s="104" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D56" s="105"/>
       <c r="E56" s="103"/>
@@ -28617,7 +28643,7 @@
       <c r="A57" s="97"/>
       <c r="B57" s="107"/>
       <c r="C57" s="104" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D57" s="105"/>
       <c r="E57" s="103"/>
@@ -28671,7 +28697,7 @@
         <v>15</v>
       </c>
       <c r="C58" s="104" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D58" s="105"/>
       <c r="E58" s="103"/>
@@ -28725,7 +28751,7 @@
       <c r="A59" s="97"/>
       <c r="B59" s="127"/>
       <c r="C59" s="104" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D59" s="105"/>
       <c r="E59" s="103"/>
@@ -28777,7 +28803,7 @@
       <c r="A60" s="97"/>
       <c r="B60" s="127"/>
       <c r="C60" s="104" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D60" s="105"/>
       <c r="E60" s="103"/>
@@ -28829,7 +28855,7 @@
       <c r="A61" s="97"/>
       <c r="B61" s="127"/>
       <c r="C61" s="128" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D61" s="129"/>
       <c r="E61" s="130"/>
@@ -28879,13 +28905,13 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="97" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B62" s="132" t="n">
         <v>16</v>
       </c>
       <c r="C62" s="104" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D62" s="105"/>
       <c r="E62" s="103"/>
@@ -28904,7 +28930,7 @@
       <c r="R62" s="103"/>
       <c r="S62" s="103"/>
       <c r="T62" s="103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U62" s="103" t="n">
         <v>0</v>
@@ -28936,7 +28962,7 @@
       <c r="A63" s="97"/>
       <c r="B63" s="132"/>
       <c r="C63" s="104" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D63" s="105"/>
       <c r="E63" s="103"/>
@@ -28955,7 +28981,7 @@
       <c r="R63" s="103"/>
       <c r="S63" s="103"/>
       <c r="T63" s="103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U63" s="103" t="n">
         <v>0</v>
@@ -28987,7 +29013,7 @@
       <c r="A64" s="97"/>
       <c r="B64" s="132"/>
       <c r="C64" s="104" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D64" s="105"/>
       <c r="E64" s="103"/>
@@ -29006,7 +29032,7 @@
       <c r="R64" s="103"/>
       <c r="S64" s="103"/>
       <c r="T64" s="103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U64" s="103" t="n">
         <v>0</v>
@@ -29038,7 +29064,7 @@
       <c r="A65" s="97"/>
       <c r="B65" s="132"/>
       <c r="C65" s="104" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="D65" s="105"/>
       <c r="E65" s="103"/>
@@ -29057,7 +29083,7 @@
       <c r="R65" s="103"/>
       <c r="S65" s="103"/>
       <c r="T65" s="103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U65" s="103" t="n">
         <v>0</v>
@@ -29091,7 +29117,7 @@
         <v>17</v>
       </c>
       <c r="C66" s="104" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D66" s="105"/>
       <c r="E66" s="103"/>
@@ -29110,7 +29136,7 @@
       <c r="R66" s="103"/>
       <c r="S66" s="103"/>
       <c r="T66" s="103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U66" s="103" t="n">
         <v>0</v>
@@ -29142,7 +29168,7 @@
       <c r="A67" s="97"/>
       <c r="B67" s="107"/>
       <c r="C67" s="104" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="D67" s="105"/>
       <c r="E67" s="103"/>
@@ -29161,7 +29187,7 @@
       <c r="R67" s="103"/>
       <c r="S67" s="103"/>
       <c r="T67" s="103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U67" s="103" t="n">
         <v>0</v>
@@ -29193,7 +29219,7 @@
       <c r="A68" s="97"/>
       <c r="B68" s="107"/>
       <c r="C68" s="104" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D68" s="105"/>
       <c r="E68" s="103"/>
@@ -29212,7 +29238,7 @@
       <c r="R68" s="103"/>
       <c r="S68" s="103"/>
       <c r="T68" s="103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U68" s="103" t="n">
         <v>0</v>
@@ -29244,7 +29270,7 @@
       <c r="A69" s="97"/>
       <c r="B69" s="107"/>
       <c r="C69" s="104" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D69" s="105"/>
       <c r="E69" s="103"/>
@@ -29263,7 +29289,7 @@
       <c r="R69" s="103"/>
       <c r="S69" s="103"/>
       <c r="T69" s="103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U69" s="103" t="n">
         <v>0</v>
@@ -29297,7 +29323,7 @@
         <v>18</v>
       </c>
       <c r="C70" s="104" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D70" s="105"/>
       <c r="E70" s="103"/>
@@ -29316,7 +29342,7 @@
       <c r="R70" s="103"/>
       <c r="S70" s="103"/>
       <c r="T70" s="103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U70" s="103" t="n">
         <v>0</v>
@@ -29348,7 +29374,7 @@
       <c r="A71" s="97"/>
       <c r="B71" s="107"/>
       <c r="C71" s="104" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="D71" s="105"/>
       <c r="E71" s="103"/>
@@ -29367,7 +29393,7 @@
       <c r="R71" s="103"/>
       <c r="S71" s="103"/>
       <c r="T71" s="103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U71" s="103" t="n">
         <v>0</v>
@@ -29399,7 +29425,7 @@
       <c r="A72" s="97"/>
       <c r="B72" s="107"/>
       <c r="C72" s="104" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="D72" s="105"/>
       <c r="E72" s="103"/>
@@ -29418,7 +29444,7 @@
       <c r="R72" s="103"/>
       <c r="S72" s="103"/>
       <c r="T72" s="103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U72" s="103" t="n">
         <v>0</v>
@@ -29450,7 +29476,7 @@
       <c r="A73" s="97"/>
       <c r="B73" s="107"/>
       <c r="C73" s="104" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="D73" s="105"/>
       <c r="E73" s="103"/>
@@ -29469,7 +29495,7 @@
       <c r="R73" s="103"/>
       <c r="S73" s="103"/>
       <c r="T73" s="103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U73" s="103" t="n">
         <v>0</v>
@@ -29503,7 +29529,7 @@
         <v>19</v>
       </c>
       <c r="C74" s="104" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D74" s="105"/>
       <c r="E74" s="103"/>
@@ -29522,7 +29548,7 @@
       <c r="R74" s="103"/>
       <c r="S74" s="103"/>
       <c r="T74" s="103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U74" s="103" t="n">
         <v>0</v>
@@ -29554,7 +29580,7 @@
       <c r="A75" s="97"/>
       <c r="B75" s="127"/>
       <c r="C75" s="104" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="D75" s="105"/>
       <c r="E75" s="103"/>
@@ -29573,7 +29599,7 @@
       <c r="R75" s="103"/>
       <c r="S75" s="103"/>
       <c r="T75" s="103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U75" s="103" t="n">
         <v>0</v>
@@ -29605,7 +29631,7 @@
       <c r="A76" s="97"/>
       <c r="B76" s="127"/>
       <c r="C76" s="104" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D76" s="105"/>
       <c r="E76" s="103"/>
@@ -29624,7 +29650,7 @@
       <c r="R76" s="103"/>
       <c r="S76" s="103"/>
       <c r="T76" s="103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U76" s="103" t="n">
         <v>0</v>
@@ -29656,7 +29682,7 @@
       <c r="A77" s="97"/>
       <c r="B77" s="127"/>
       <c r="C77" s="128" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D77" s="129"/>
       <c r="E77" s="130"/>
@@ -29675,7 +29701,7 @@
       <c r="R77" s="130"/>
       <c r="S77" s="130"/>
       <c r="T77" s="130" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="U77" s="130" t="n">
         <v>0</v>
@@ -29842,7 +29868,7 @@
       <c r="A80" s="103"/>
       <c r="B80" s="103"/>
       <c r="C80" s="137" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="D80" s="137"/>
       <c r="E80" s="102" t="n">
@@ -29868,7 +29894,7 @@
       <c r="W80" s="103"/>
       <c r="X80" s="103"/>
       <c r="Y80" s="138" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="Z80" s="103"/>
       <c r="AA80" s="103"/>
@@ -29884,7 +29910,7 @@
       <c r="A81" s="103"/>
       <c r="B81" s="103"/>
       <c r="C81" s="139" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="D81" s="139"/>
       <c r="E81" s="106" t="n">
@@ -29924,7 +29950,7 @@
       <c r="A82" s="103"/>
       <c r="B82" s="103"/>
       <c r="C82" s="139" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D82" s="139"/>
       <c r="E82" s="106" t="n">
@@ -29964,7 +29990,7 @@
       <c r="A83" s="103"/>
       <c r="B83" s="103"/>
       <c r="C83" s="139" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D83" s="139"/>
       <c r="E83" s="106" t="n">
@@ -30004,7 +30030,7 @@
       <c r="A84" s="103"/>
       <c r="B84" s="103"/>
       <c r="C84" s="139" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="D84" s="139"/>
       <c r="E84" s="106" t="n">
@@ -30044,7 +30070,7 @@
       <c r="A85" s="103"/>
       <c r="B85" s="103"/>
       <c r="C85" s="140" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="D85" s="140"/>
       <c r="E85" s="131" t="n">
@@ -30168,98 +30194,98 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="42" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B4" s="141" t="n">
         <v>43739</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B5" s="141" t="n">
         <v>44621</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B6" s="142" t="n">
         <f aca="false">B5-B4</f>
         <v>882</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B7" s="143" t="n">
         <f aca="false">B6/365</f>
         <v>2.41643835616438</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B8" s="144" t="n">
         <v>7.5</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="42" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C10" s="145" t="n">
         <f aca="false">260*B8*0.2*B7</f>
         <v>942.41095890411</v>
       </c>
       <c r="F10" s="146" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F11" s="146" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="42" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C12" s="147" t="e">
         <f aca="false">'otjt log'!#ref!</f>
         <v>#VALUE!</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="42" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C14" s="148" t="e">
         <f aca="false">C12-C10</f>
@@ -30268,7 +30294,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="149" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>
@@ -30321,7 +30347,7 @@
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
       <c r="B2" s="150" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C2" s="151"/>
       <c r="D2" s="151"/>
@@ -30344,7 +30370,7 @@
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2"/>
       <c r="B3" s="153" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C3" s="154"/>
       <c r="D3" s="154"/>
@@ -30367,7 +30393,7 @@
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2"/>
       <c r="B4" s="155" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C4" s="154"/>
       <c r="D4" s="154"/>
@@ -30390,7 +30416,7 @@
     <row r="5" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2"/>
       <c r="B5" s="156" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C5" s="156"/>
       <c r="D5" s="156"/>
@@ -30413,7 +30439,7 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2"/>
       <c r="B6" s="157" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C6" s="157"/>
       <c r="D6" s="157"/>
@@ -30484,7 +30510,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="163" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>